<commit_message>
Great progress in chapters 1, 2 and 3.
</commit_message>
<xml_diff>
--- a/diagramas/Gantt.xlsx
+++ b/diagramas/Gantt.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ricardo\Desktop\Tese_mestrado\diagramas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E7051B8-73B8-482F-A6AC-D57E059E31AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F09862B-8473-4278-89C4-FCBB73B594E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{9E5D4881-DCE1-478A-8E87-A90D197304B3}"/>
   </bookViews>
@@ -37,93 +37,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Ano</t>
-  </si>
-  <si>
-    <t>Start Date</t>
-  </si>
-  <si>
-    <t>Days Needed</t>
-  </si>
-  <si>
-    <t>Completion</t>
-  </si>
-  <si>
-    <t>CRT+1</t>
-  </si>
-  <si>
-    <t>Men</t>
-  </si>
-  <si>
-    <t>d</t>
-  </si>
-  <si>
-    <t>f</t>
-  </si>
-  <si>
-    <t>df</t>
-  </si>
-  <si>
-    <t>ad</t>
-  </si>
-  <si>
-    <t>adf</t>
-  </si>
-  <si>
-    <t>gv</t>
-  </si>
-  <si>
-    <t>cx</t>
-  </si>
-  <si>
-    <t>ba</t>
-  </si>
-  <si>
-    <t>vret</t>
-  </si>
-  <si>
-    <t>ywrty</t>
-  </si>
-  <si>
-    <t>u</t>
-  </si>
-  <si>
-    <t>lio</t>
-  </si>
-  <si>
-    <t>waecew</t>
-  </si>
-  <si>
-    <t>re</t>
-  </si>
-  <si>
-    <t>er</t>
-  </si>
-  <si>
-    <t>eqrfer</t>
-  </si>
-  <si>
-    <t>ref</t>
-  </si>
-  <si>
-    <t>erf</t>
-  </si>
-  <si>
-    <t>iopç</t>
   </si>
   <si>
     <t>Nivel</t>
   </si>
   <si>
     <t>Label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sdf </t>
-  </si>
-  <si>
-    <t>Adjusted Length</t>
   </si>
   <si>
     <t>Tarefas</t>
@@ -138,19 +60,40 @@
     <t>Implementação do simulated annealing</t>
   </si>
   <si>
-    <t>Implementação do parser dos dados ITC 2019</t>
-  </si>
-  <si>
     <t>Implementação da interface gráfica</t>
   </si>
   <si>
     <t>Avaliação e correção da aplicação</t>
+  </si>
+  <si>
+    <t>Data de inicio</t>
+  </si>
+  <si>
+    <t>Data de fim</t>
+  </si>
+  <si>
+    <t>Implementação da base de dados</t>
+  </si>
+  <si>
+    <t>Duração (dias)</t>
+  </si>
+  <si>
+    <t>Duração (semanas)</t>
+  </si>
+  <si>
+    <t>Conversão dos dados de entrada para o padrão ITC 2019</t>
+  </si>
+  <si>
+    <t>Implementação do interpretador dos dados ITC 2019</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="170" formatCode="0.0"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -186,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -202,6 +145,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -234,36 +186,6 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="pt-PT"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
@@ -280,7 +202,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Start Date</c:v>
+                  <c:v>Data de inicio</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -295,22 +217,28 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>GANTT!$A$3:$A$8</c:f>
+              <c:f>GANTT!$A$3:$A$9</c:f>
               <c:strCache>
-                <c:ptCount val="6"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>Escrita do TFM</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>Conversão dos dados de entrada para o padrão ITC 2019</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Implementação do interpretador dos dados ITC 2019</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Implementação da base de dados</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>Implementação do simulated annealing</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>Implementação do parser dos dados ITC 2019</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>Implementação da interface gráfica</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>Avaliação e correção da aplicação</c:v>
                 </c:pt>
               </c:strCache>
@@ -318,31 +246,37 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>GANTT!$B$3:$B$8</c:f>
+              <c:f>GANTT!$B$3:$B$9</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>45658</c:v>
+                  <c:v>45717</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>45717</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>45762</c:v>
+                  <c:v>45722</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>45736</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>45757</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>45787</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>45828</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-4CC2-4647-A678-764D53F39475}"/>
+              <c16:uniqueId val="{00000000-EA04-4B3F-96C6-E2A752F8A4AF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -351,11 +285,11 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>GANTT!$E$2</c:f>
+              <c:f>GANTT!$D$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Adjusted Length</c:v>
+                  <c:v>Duração (dias)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -372,22 +306,28 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>GANTT!$A$3:$A$8</c:f>
+              <c:f>GANTT!$A$3:$A$9</c:f>
               <c:strCache>
-                <c:ptCount val="6"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>Escrita do TFM</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>Conversão dos dados de entrada para o padrão ITC 2019</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Implementação do interpretador dos dados ITC 2019</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Implementação da base de dados</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>Implementação do simulated annealing</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>Implementação do parser dos dados ITC 2019</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>Implementação da interface gráfica</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>Avaliação e correção da aplicação</c:v>
                 </c:pt>
               </c:strCache>
@@ -395,31 +335,37 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>GANTT!$E$3:$E$8</c:f>
+              <c:f>GANTT!$D$3:$D$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>213</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>21</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>41</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>11</c:v>
+                <c:pt idx="6">
+                  <c:v>73</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4CC2-4647-A678-764D53F39475}"/>
+              <c16:uniqueId val="{00000001-EA04-4B3F-96C6-E2A752F8A4AF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -433,11 +379,11 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="1897605695"/>
-        <c:axId val="1897606527"/>
+        <c:axId val="472744224"/>
+        <c:axId val="472743744"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1897605695"/>
+        <c:axId val="472744224"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -480,7 +426,7 @@
             <a:endParaRPr lang="pt-PT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1897606527"/>
+        <c:crossAx val="472743744"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -488,10 +434,10 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1897606527"/>
+        <c:axId val="472743744"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="45798"/>
+          <c:max val="45930"/>
           <c:min val="45717"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -510,6 +456,20 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="5000"/>
+                  <a:lumOff val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:minorGridlines>
         <c:numFmt formatCode="m/d/yyyy" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -517,16 +477,21 @@
         <c:spPr>
           <a:noFill/>
           <a:ln>
-            <a:noFill/>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
         <c:txPr>
-          <a:bodyPr rot="-2700000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -541,10 +506,10 @@
             <a:endParaRPr lang="pt-PT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1897605695"/>
+        <c:crossAx val="472744224"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
-        <c:majorUnit val="7"/>
+        <c:majorUnit val="26.625"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -554,37 +519,6 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="pt-PT"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:extLst>
@@ -655,7 +589,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Folha2!$C$2</c:f>
+              <c:f>Folha2!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -680,7 +614,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F9CD0CC4-0984-4D9B-8F3F-A1C9DC4CDF15}" type="CELLRANGE">
+                    <a:fld id="{81E75F69-ADC0-42BB-87D7-BEE35BCFA4F4}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -713,8 +647,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{4BF565E3-4DBE-4076-96FB-E7968589EDD7}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{4C7FD7FC-901E-495B-B613-AB65D10B551C}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -732,6 +666,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -746,8 +681,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F11A2811-DBE7-4500-8A76-F1B334FABF8C}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{16B83809-4D41-45B0-B1A7-795B9966D3D3}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -765,6 +700,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -779,8 +715,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{0EEC4882-76DA-4A45-A9F7-8282866940B7}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{8A1A5C0A-6A45-4159-A770-6A6A89E17A0E}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -798,6 +734,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -812,8 +749,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E394C691-45BD-4C44-A877-B5FB877454E4}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{8D3766C9-A2F9-4B57-973D-EF66C8B3F037}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -831,6 +768,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -845,8 +783,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E4C3FD44-4461-4387-AFE8-961B35C1115A}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{6F554FF5-A235-4E5F-8EC3-F6FB60283B4A}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -864,6 +802,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -878,8 +817,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AE82EDDD-9F61-4020-9750-CF7E4E2E2EF5}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{180499CC-8A71-4089-ADA2-B9B026E4C3E9}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -897,6 +836,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -911,8 +851,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FFCCE442-BB03-4DBA-B1FF-D0E6503B7BEB}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{35AF636C-1C9B-44AC-AF2A-39171CBCAABE}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -930,6 +870,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -944,8 +885,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{525E8825-CD4F-490E-9E65-C0F006300FC1}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{DB819A59-A9DC-45D3-B4FD-935645DDAAAC}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -963,6 +904,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -977,8 +919,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D73D920F-5FAF-45B4-83EA-C2D35F5DA198}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{7A49A243-0C2F-4FFE-A8AB-D1D7BD3C4535}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -996,6 +938,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1010,8 +953,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E6C35E39-A094-4AAB-9545-B2A976CDF22D}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{BEBEEC8E-3C68-427C-8946-DDA8FCE8B035}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1029,6 +972,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1043,8 +987,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FE1FD09F-1186-4151-B96B-ACED0B24C8AF}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{7C043B7E-837E-49AE-B272-08A27E6EFC03}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1062,6 +1006,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1076,8 +1021,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C5C2F398-6B1A-4560-A914-7FE4D3B4ABBB}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{7D1247E9-C7D1-431D-A655-3218C3089820}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1095,6 +1040,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1109,8 +1055,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{95313948-481C-4471-9386-AA9D3FDC7943}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{A0E6D1D0-AC34-46BA-93B9-9B0A751F2795}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1128,6 +1074,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1142,8 +1089,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{02C15113-F760-49C0-8E34-8137797A744B}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{CA2CF1D4-4290-44E4-AE8D-61890CDA4A93}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1161,6 +1108,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1175,8 +1123,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F2677B4B-FF85-42E5-9EDF-265503547153}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{06532B60-726B-47CE-93B2-B84D41F1AFAB}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1194,6 +1142,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1208,8 +1157,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{026E0982-04F5-4640-A0FA-6A93CB6BCAEE}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{8E5257A3-A761-4DEE-8EC7-A239488A7EA3}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1227,6 +1176,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1241,8 +1191,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{76F64FEC-42EE-454C-AD1D-5B72594F460A}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{FAE214F6-788A-4020-A5C7-BD79D5D29688}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1260,6 +1210,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1274,8 +1225,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{203AF54C-F89E-4EEE-A9D1-BE58A25A6670}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{53451286-C5FB-4B34-BE0F-7E4325DC4D13}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1293,6 +1244,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1307,8 +1259,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{0D47A660-E564-49A9-9984-EDC43A2D1913}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{4FEE6517-CFD8-48E6-9B11-E39E7CAFDB4F}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1326,6 +1278,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1340,8 +1293,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9B505E77-8C35-4F39-84BB-90CA6CB51248}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{5156A5FD-1FC4-475D-8EB9-DB0206378B83}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1359,6 +1312,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1373,8 +1327,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{B0727477-2C24-49F1-8D4C-A4CBF891CACD}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{65C33C34-3371-4FCB-970E-00E7FA3B82CD}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1392,6 +1346,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1406,8 +1361,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{DBDFE10A-D330-4E0C-9ADA-A42580938AF3}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{227DB3BA-0A8C-47E7-AC70-67117EDAB765}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1425,6 +1380,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1439,8 +1395,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3F55B415-9140-455A-B875-3D05C4E67F6E}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{85BC8113-FEB3-4F49-A64A-7EC6715D7E0D}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1458,6 +1414,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1472,8 +1429,8 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6FF3CDB8-99F5-47DF-A804-B477D0AC617F}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
+                    <a:fld id="{18AB1DBE-5D9B-4943-9614-B8549A729B35}" type="CELLRANGE">
+                      <a:rPr lang="pt-PT"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
                     </a:fld>
@@ -1491,6 +1448,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
+                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1574,7 +1532,7 @@
           </c:errBars>
           <c:cat>
             <c:numRef>
-              <c:f>Folha2!$B$3:$B$27</c:f>
+              <c:f>Folha2!$A$2:$A$26</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
                 <c:ptCount val="25"/>
@@ -1658,7 +1616,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Folha2!$C$3:$C$27</c:f>
+              <c:f>Folha2!$B$2:$B$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="25"/>
@@ -1743,7 +1701,7 @@
           <c:extLst>
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
               <c15:datalabelsRange>
-                <c15:f>Folha2!$D$3:$D$27</c15:f>
+                <c15:f>Folha2!$C$2:$C$26</c15:f>
                 <c15:dlblRangeCache>
                   <c:ptCount val="25"/>
                 </c15:dlblRangeCache>
@@ -2966,23 +2924,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>273050</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>495299</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>14287</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>90487</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Gráfico 4">
+        <xdr:cNvPr id="2" name="Gráfico 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E64627C5-E4C5-9F43-AADE-3B681128A194}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BC5F87D5-2B92-D96A-21D8-22C5960D494A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3341,156 +3299,189 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BF3AA6B-9DCA-46B7-9978-7DB82B4E0B9C}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="41.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
       <c r="E1" s="5"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="B3" s="2">
-        <v>45658</v>
-      </c>
-      <c r="C3" s="1">
-        <v>15</v>
-      </c>
-      <c r="D3" s="2">
-        <f>WORKDAY(B3,C3)</f>
-        <v>45679</v>
-      </c>
-      <c r="E3" s="1">
-        <f>D3-B3</f>
-        <v>21</v>
-      </c>
+        <v>45717</v>
+      </c>
+      <c r="C3" s="2">
+        <v>45930</v>
+      </c>
+      <c r="D3" s="1">
+        <f>C3-B3</f>
+        <v>213</v>
+      </c>
+      <c r="E3" s="7">
+        <f>D3/7</f>
+        <v>30.428571428571427</v>
+      </c>
+      <c r="G3" s="8"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2">
         <v>45717</v>
       </c>
-      <c r="C4" s="1">
-        <v>30</v>
-      </c>
-      <c r="D4" s="2">
-        <f t="shared" ref="D4:D8" si="0">WORKDAY(B4,C4)</f>
-        <v>45758</v>
-      </c>
-      <c r="E4" s="1">
-        <f t="shared" ref="E4:E8" si="1">D4-B4</f>
-        <v>41</v>
-      </c>
+      <c r="C4" s="2">
+        <v>45724</v>
+      </c>
+      <c r="D4" s="1">
+        <f t="shared" ref="D4:D8" si="0">C4-B4</f>
+        <v>7</v>
+      </c>
+      <c r="E4" s="7">
+        <f t="shared" ref="E4:E9" si="1">D4/7</f>
+        <v>1</v>
+      </c>
+      <c r="G4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="B5" s="2">
-        <v>45762</v>
-      </c>
-      <c r="C5" s="1">
-        <v>5</v>
-      </c>
-      <c r="D5" s="2">
-        <f t="shared" si="0"/>
-        <v>45769</v>
-      </c>
-      <c r="E5" s="1">
+        <v>45722</v>
+      </c>
+      <c r="C5" s="2">
+        <v>45743</v>
+      </c>
+      <c r="D5" s="1">
+        <f>C5-B5</f>
+        <v>21</v>
+      </c>
+      <c r="E5" s="7">
         <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="G5" s="8"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="2">
+        <v>45736</v>
+      </c>
+      <c r="C6" s="2">
+        <v>45757</v>
+      </c>
+      <c r="D6" s="1">
+        <f>C6-B6</f>
+        <v>21</v>
+      </c>
+      <c r="E6" s="7">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="G6" s="8"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>45757</v>
+      </c>
+      <c r="C7" s="2">
+        <v>45785</v>
+      </c>
+      <c r="D7" s="1">
+        <f>C7-B7</f>
+        <v>28</v>
+      </c>
+      <c r="E7" s="7">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="G7" s="8"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="2">
-        <v>45757</v>
-      </c>
-      <c r="C6" s="1">
-        <v>10</v>
-      </c>
-      <c r="D6" s="2">
-        <f t="shared" si="0"/>
-        <v>45771</v>
-      </c>
-      <c r="E6" s="1">
-        <f t="shared" si="1"/>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="2"/>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="B8" s="2">
         <v>45787</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="2">
+        <v>45828</v>
+      </c>
+      <c r="D8" s="1">
+        <f>C8-B8</f>
+        <v>41</v>
+      </c>
+      <c r="E8" s="7">
+        <f t="shared" si="1"/>
+        <v>5.8571428571428568</v>
+      </c>
+      <c r="G8" s="8"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="2">
-        <f t="shared" si="0"/>
-        <v>45798</v>
-      </c>
-      <c r="E8" s="1">
+      <c r="B9" s="2">
+        <v>45828</v>
+      </c>
+      <c r="C9" s="2">
+        <v>45901</v>
+      </c>
+      <c r="D9" s="1">
+        <f>C9-B9</f>
+        <v>73</v>
+      </c>
+      <c r="E9" s="7">
         <f t="shared" si="1"/>
-        <v>11</v>
-      </c>
+        <v>10.428571428571429</v>
+      </c>
+      <c r="G9" s="8"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C9" s="1">
-        <f>SUM(C3:C8)</f>
-        <v>68</v>
-      </c>
-      <c r="E9" s="1">
-        <f>SUM(E3:E8)</f>
-        <v>94</v>
-      </c>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="1" t="s">
-        <v>4</v>
-      </c>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3504,327 +3495,274 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2C88C66-FB8F-439A-AAB7-DE57B87D878E}">
-  <dimension ref="A2:D27"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" style="1"/>
-    <col min="4" max="4" width="13.42578125" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>26</v>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>36526</v>
       </c>
-      <c r="C3" s="1">
+      <c r="B2" s="1">
         <v>2</v>
       </c>
+      <c r="C2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2">
-        <f>B3+366</f>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <f>A2+366</f>
         <v>36892</v>
       </c>
-      <c r="C4" s="1">
+      <c r="B3" s="1">
         <v>-2</v>
       </c>
+      <c r="C3"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="2">
-        <f>B4+365</f>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <f>A3+365</f>
         <v>37257</v>
       </c>
-      <c r="C5" s="1">
+      <c r="B4" s="1">
         <v>4</v>
       </c>
+      <c r="C4"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="2">
-        <f>B5+365</f>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <f>A4+365</f>
         <v>37622</v>
       </c>
-      <c r="C6" s="1">
+      <c r="B5" s="1">
         <v>-4</v>
       </c>
+      <c r="C5"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2">
-        <f t="shared" ref="B7:B27" si="0">B6+365</f>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <f t="shared" ref="A6:A26" si="0">A5+365</f>
         <v>37987</v>
       </c>
-      <c r="C7" s="1">
+      <c r="B6" s="1">
         <v>2</v>
       </c>
+      <c r="C6"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2">
-        <f>B7+366</f>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <f>A6+366</f>
         <v>38353</v>
       </c>
-      <c r="C8" s="1">
+      <c r="B7" s="1">
         <v>-2</v>
       </c>
+      <c r="C7"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
         <f t="shared" si="0"/>
         <v>38718</v>
       </c>
-      <c r="C9" s="1">
+      <c r="B8" s="1">
         <v>4</v>
       </c>
+      <c r="C8"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
         <f t="shared" si="0"/>
         <v>39083</v>
       </c>
-      <c r="C10" s="1">
+      <c r="B9" s="1">
         <v>-4</v>
       </c>
+      <c r="C9"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
         <f t="shared" si="0"/>
         <v>39448</v>
       </c>
-      <c r="C11" s="1">
+      <c r="B10" s="1">
         <v>2</v>
       </c>
+      <c r="C10"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" s="2">
-        <f>B11+366</f>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <f>A10+366</f>
         <v>39814</v>
       </c>
-      <c r="C12" s="1">
+      <c r="B11" s="1">
         <v>-2</v>
       </c>
+      <c r="C11"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
         <f t="shared" si="0"/>
         <v>40179</v>
       </c>
-      <c r="C13" s="1">
+      <c r="B12" s="1">
         <v>4</v>
       </c>
+      <c r="C12"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
         <f t="shared" si="0"/>
         <v>40544</v>
       </c>
-      <c r="C14" s="1">
+      <c r="B13" s="1">
         <v>-4</v>
       </c>
+      <c r="C13"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
         <f t="shared" si="0"/>
         <v>40909</v>
       </c>
-      <c r="C15" s="1">
+      <c r="B14" s="1">
         <v>2</v>
       </c>
+      <c r="C14"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="2">
-        <f>B15+366</f>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <f>A14+366</f>
         <v>41275</v>
       </c>
-      <c r="C16" s="1">
+      <c r="B15" s="1">
         <v>-2</v>
       </c>
+      <c r="C15"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <f t="shared" si="0"/>
+        <v>41640</v>
+      </c>
+      <c r="B16" s="1">
+        <v>4</v>
+      </c>
+      <c r="C16"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" s="2">
+      <c r="A17" s="2">
         <f t="shared" si="0"/>
-        <v>41640</v>
-      </c>
-      <c r="C17" s="1">
-        <v>4</v>
-      </c>
+        <v>42005</v>
+      </c>
+      <c r="B17" s="1">
+        <v>-4</v>
+      </c>
+      <c r="C17"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" s="2">
+      <c r="A18" s="2">
         <f t="shared" si="0"/>
-        <v>42005</v>
-      </c>
-      <c r="C18" s="1">
-        <v>-4</v>
-      </c>
+        <v>42370</v>
+      </c>
+      <c r="B18" s="1">
+        <v>2</v>
+      </c>
+      <c r="C18"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B19" s="2">
-        <f t="shared" si="0"/>
-        <v>42370</v>
-      </c>
-      <c r="C19" s="1">
-        <v>2</v>
-      </c>
+      <c r="A19" s="2">
+        <f>A18+366</f>
+        <v>42736</v>
+      </c>
+      <c r="B19" s="1">
+        <v>-2</v>
+      </c>
+      <c r="C19"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B20" s="2">
-        <f>B19+366</f>
-        <v>42736</v>
-      </c>
-      <c r="C20" s="1">
-        <v>-2</v>
-      </c>
+      <c r="A20" s="2">
+        <f t="shared" si="0"/>
+        <v>43101</v>
+      </c>
+      <c r="B20" s="1">
+        <v>4</v>
+      </c>
+      <c r="C20"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B21" s="2">
+      <c r="A21" s="2">
         <f t="shared" si="0"/>
-        <v>43101</v>
-      </c>
-      <c r="C21" s="1">
-        <v>4</v>
-      </c>
+        <v>43466</v>
+      </c>
+      <c r="B21" s="1">
+        <v>-4</v>
+      </c>
+      <c r="C21"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="2">
+      <c r="A22" s="2">
         <f t="shared" si="0"/>
-        <v>43466</v>
-      </c>
-      <c r="C22" s="1">
-        <v>-4</v>
-      </c>
+        <v>43831</v>
+      </c>
+      <c r="B22" s="1">
+        <v>2</v>
+      </c>
+      <c r="C22"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B23" s="2">
-        <f t="shared" si="0"/>
-        <v>43831</v>
-      </c>
-      <c r="C23" s="1">
-        <v>2</v>
-      </c>
+      <c r="A23" s="2">
+        <f>A22+366</f>
+        <v>44197</v>
+      </c>
+      <c r="B23" s="1">
+        <v>-2</v>
+      </c>
+      <c r="C23"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B24" s="2">
-        <f>B23+366</f>
-        <v>44197</v>
-      </c>
-      <c r="C24" s="1">
-        <v>-2</v>
-      </c>
+      <c r="A24" s="2">
+        <f t="shared" si="0"/>
+        <v>44562</v>
+      </c>
+      <c r="B24" s="1">
+        <v>4</v>
+      </c>
+      <c r="C24"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" s="2">
+      <c r="A25" s="2">
         <f t="shared" si="0"/>
-        <v>44562</v>
-      </c>
-      <c r="C25" s="1">
-        <v>4</v>
-      </c>
+        <v>44927</v>
+      </c>
+      <c r="B25" s="1">
+        <v>-4</v>
+      </c>
+      <c r="C25"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" s="2">
-        <f t="shared" si="0"/>
-        <v>44927</v>
-      </c>
-      <c r="C26" s="1">
-        <v>-4</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B27" s="2">
+      <c r="A26" s="2">
         <f t="shared" si="0"/>
         <v>45292</v>
       </c>
-      <c r="C27" s="1">
+      <c r="B26" s="1">
         <v>2</v>
       </c>
+      <c r="C26"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Continuation of the writing of the thesis. Start of the creation of the database.
</commit_message>
<xml_diff>
--- a/diagramas/Gantt.xlsx
+++ b/diagramas/Gantt.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ricardo\Desktop\Tese_mestrado\diagramas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F09862B-8473-4278-89C4-FCBB73B594E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BCE4E19-1244-4E79-9551-56274FAD60A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{9E5D4881-DCE1-478A-8E87-A90D197304B3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{9E5D4881-DCE1-478A-8E87-A90D197304B3}"/>
   </bookViews>
   <sheets>
     <sheet name="GANTT" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Ano</t>
   </si>
@@ -86,13 +86,16 @@
   <si>
     <t>Implementação do interpretador dos dados ITC 2019</t>
   </si>
+  <si>
+    <t>Planeamento da arquitetura</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -129,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -143,17 +146,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -217,28 +217,31 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>GANTT!$A$3:$A$9</c:f>
+              <c:f>GANTT!$A$3:$A$10</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>Escrita do TFM</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>Planeamento da arquitetura</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>Conversão dos dados de entrada para o padrão ITC 2019</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>Implementação do interpretador dos dados ITC 2019</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>Implementação da base de dados</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>Implementação do simulated annealing</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>Implementação da interface gráfica</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>Avaliação e correção da aplicação</c:v>
                 </c:pt>
               </c:strCache>
@@ -246,10 +249,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>GANTT!$B$3:$B$9</c:f>
+              <c:f>GANTT!$B$3:$B$10</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>45717</c:v>
                 </c:pt>
@@ -257,18 +260,21 @@
                   <c:v>45717</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>45717</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>45722</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>45736</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>45757</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>45787</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>45828</c:v>
                 </c:pt>
               </c:numCache>
@@ -306,28 +312,31 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>GANTT!$A$3:$A$9</c:f>
+              <c:f>GANTT!$A$3:$A$10</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>Escrita do TFM</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>Planeamento da arquitetura</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>Conversão dos dados de entrada para o padrão ITC 2019</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>Implementação do interpretador dos dados ITC 2019</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>Implementação da base de dados</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>Implementação do simulated annealing</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>Implementação da interface gráfica</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>Avaliação e correção da aplicação</c:v>
                 </c:pt>
               </c:strCache>
@@ -335,10 +344,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>GANTT!$D$3:$D$9</c:f>
+              <c:f>GANTT!$D$3:$D$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>213</c:v>
                 </c:pt>
@@ -346,18 +355,21 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>21</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>28</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>41</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>73</c:v>
                 </c:pt>
               </c:numCache>
@@ -614,7 +626,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{81E75F69-ADC0-42BB-87D7-BEE35BCFA4F4}" type="CELLRANGE">
+                    <a:fld id="{D5E2CF66-DCAB-4B5A-AACA-2B695081D6EB}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[INTERVALODACÉLULA]</a:t>
@@ -666,7 +678,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -700,7 +711,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -734,7 +744,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -768,7 +777,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -802,7 +810,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -836,7 +843,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -870,7 +876,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -904,7 +909,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -938,7 +942,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -972,7 +975,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1006,7 +1008,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1040,7 +1041,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1074,7 +1074,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1108,7 +1107,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1142,7 +1140,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1176,7 +1173,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1210,7 +1206,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1244,7 +1239,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1278,7 +1272,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1312,7 +1305,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1346,7 +1338,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1380,7 +1371,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1414,7 +1404,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1448,7 +1437,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -2925,15 +2913,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>495299</xdr:colOff>
+      <xdr:colOff>476249</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>14287</xdr:rowOff>
+      <xdr:rowOff>166687</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
+      <xdr:colOff>114300</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>90487</xdr:rowOff>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3299,7 +3287,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BF3AA6B-9DCA-46B7-9978-7DB82B4E0B9C}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51" style="1" bestFit="1" customWidth="1"/>
@@ -3311,13 +3299,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -3350,15 +3338,15 @@
         <f>C3-B3</f>
         <v>213</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="5">
         <f>D3/7</f>
         <v>30.428571428571427</v>
       </c>
-      <c r="G3" s="8"/>
+      <c r="G3" s="6"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2">
         <v>45717</v>
@@ -3367,121 +3355,133 @@
         <v>45724</v>
       </c>
       <c r="D4" s="1">
-        <f t="shared" ref="D4:D8" si="0">C4-B4</f>
+        <f>C4-B4</f>
         <v>7</v>
       </c>
-      <c r="E4" s="7">
-        <f t="shared" ref="E4:E9" si="1">D4/7</f>
+      <c r="E4" s="5">
+        <f>D4/7</f>
         <v>1</v>
       </c>
-      <c r="G4" s="8"/>
+      <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="2">
-        <v>45722</v>
+        <v>45717</v>
       </c>
       <c r="C5" s="2">
-        <v>45743</v>
+        <v>45724</v>
       </c>
       <c r="D5" s="1">
-        <f>C5-B5</f>
-        <v>21</v>
-      </c>
-      <c r="E5" s="7">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="G5" s="8"/>
+        <f t="shared" ref="D5" si="0">C5-B5</f>
+        <v>7</v>
+      </c>
+      <c r="E5" s="5">
+        <f t="shared" ref="E5:E10" si="1">D5/7</f>
+        <v>1</v>
+      </c>
+      <c r="G5" s="6"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B6" s="2">
-        <v>45736</v>
+        <v>45722</v>
       </c>
       <c r="C6" s="2">
-        <v>45757</v>
+        <v>45743</v>
       </c>
       <c r="D6" s="1">
         <f>C6-B6</f>
         <v>21</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="5">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="G6" s="8"/>
+      <c r="G6" s="6"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B7" s="2">
+        <v>45736</v>
+      </c>
+      <c r="C7" s="2">
         <v>45757</v>
-      </c>
-      <c r="C7" s="2">
-        <v>45785</v>
       </c>
       <c r="D7" s="1">
         <f>C7-B7</f>
-        <v>28</v>
-      </c>
-      <c r="E7" s="7">
+        <v>21</v>
+      </c>
+      <c r="E7" s="5">
         <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="G7" s="8"/>
+        <v>3</v>
+      </c>
+      <c r="G7" s="6"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="2">
-        <v>45787</v>
+        <v>45757</v>
       </c>
       <c r="C8" s="2">
-        <v>45828</v>
+        <v>45785</v>
       </c>
       <c r="D8" s="1">
         <f>C8-B8</f>
-        <v>41</v>
-      </c>
-      <c r="E8" s="7">
+        <v>28</v>
+      </c>
+      <c r="E8" s="5">
         <f t="shared" si="1"/>
-        <v>5.8571428571428568</v>
-      </c>
-      <c r="G8" s="8"/>
+        <v>4</v>
+      </c>
+      <c r="G8" s="6"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="2">
+        <v>45787</v>
+      </c>
+      <c r="C9" s="2">
         <v>45828</v>
-      </c>
-      <c r="C9" s="2">
-        <v>45901</v>
       </c>
       <c r="D9" s="1">
         <f>C9-B9</f>
+        <v>41</v>
+      </c>
+      <c r="E9" s="5">
+        <f t="shared" si="1"/>
+        <v>5.8571428571428568</v>
+      </c>
+      <c r="G9" s="6"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2">
+        <v>45828</v>
+      </c>
+      <c r="C10" s="2">
+        <v>45901</v>
+      </c>
+      <c r="D10" s="1">
+        <f>C10-B10</f>
         <v>73</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E10" s="5">
         <f t="shared" si="1"/>
         <v>10.428571428571429</v>
       </c>
-      <c r="G9" s="8"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B13" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>